<commit_message>
🔄 Auto-collect traffic data: 2026-10-17 01:19 PM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-10-17_Sat.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-10-17_Sat.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="All Periods Combined" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="1_00 PM" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="449">
   <si>
     <t>Date</t>
   </si>
@@ -122,7 +123,7 @@
     <t>12:00 AM</t>
   </si>
   <si>
-    <t>Friday (Weekday) - Night Off-Peak</t>
+    <t>Saturday (Weekend) - Night Off-Peak</t>
   </si>
   <si>
     <t>Blue Line</t>
@@ -824,6 +825,489 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/12_00_AM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>10/17/2026, 1:03:39 PM</t>
+  </si>
+  <si>
+    <t>1:00 PM</t>
+  </si>
+  <si>
+    <t>Saturday (Weekend) - Mid-day Off-Peak</t>
+  </si>
+  <si>
+    <t> | 30 min | 1:00 PM—1:30 PM | Blue Line | 1:00 PM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 1 hr 3 min | 13.3 km | via Barrackpore Trunk Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>33 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.10x</t>
+  </si>
+  <si>
+    <t>52.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:04:10 PM</t>
+  </si>
+  <si>
+    <t> | 33 min | 1:00 PM—1:33 PM | Blue Line | 1:00 PM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 1 hr 9 min | 14.7 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>36 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.09x</t>
+  </si>
+  <si>
+    <t>52.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:04:28 PM</t>
+  </si>
+  <si>
+    <t> | 54 min | 3.8 km | via Belgachia Rd/Khudiram Bose Sarani</t>
+  </si>
+  <si>
+    <t> | 23 min | 4.1 km | via Belgachia Rd/Khudiram Bose Sarani | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>31 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.43x</t>
+  </si>
+  <si>
+    <t>57.4% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:05:00 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 1:00 PM—1:11 PM | Blue Line | 1:00 PM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 39 min | 5.2 km | via Jatindra Mohan Ave and Central Ave/Chittaranjan Ave | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>28 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>3.55x</t>
+  </si>
+  <si>
+    <t>71.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:05:31 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 1:04 PM—1:15 PM | Blue Line | 1:04 PM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 23 min | 5.1 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:05:52 PM</t>
+  </si>
+  <si>
+    <t>Train Walk</t>
+  </si>
+  <si>
+    <t> | 26 min | 5:27 AM—5:53 AM | 32212 - Dankuni - Sealdah Local </t>
+  </si>
+  <si>
+    <t> | 28 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, despite slowdown on SH 1 causing 9-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.08x</t>
+  </si>
+  <si>
+    <t>7.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:06:23 PM</t>
+  </si>
+  <si>
+    <t> | 24 min | 1:11 PM—1:35 PM | Blue Line | 1:11 PM from Esplanade | ₹15.00  1 min | Details</t>
+  </si>
+  <si>
+    <t> | 35 min | 8.3 km | via Chowringee Rd/Jawaharlal Nehru Rd and Ashutosh Mukherjee Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.46x</t>
+  </si>
+  <si>
+    <t>31.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:06:57 PM</t>
+  </si>
+  <si>
+    <t> | 17 min | 12:54 PM—1:11 PM | Blue Line | 12:55 PM from Mahanayak Uttamkumar | ₹15.00  1 min | Details</t>
+  </si>
+  <si>
+    <t> | 29 min | 6.4 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.71x</t>
+  </si>
+  <si>
+    <t>41.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:07:30 PM</t>
+  </si>
+  <si>
+    <t> | 16 min | 1:00 PM—1:16 PM | Blue Line | 1:00 PM from Dumdum | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 57 min | 8.8 km | via Jessore Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>41 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>3.56x</t>
+  </si>
+  <si>
+    <t>71.9% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:08:01 PM</t>
+  </si>
+  <si>
+    <t> | 30 min | 1:32 PM—2:02 PM | Green Line | 1:32 PM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 56 min | 12.9 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>26 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.87x</t>
+  </si>
+  <si>
+    <t>46.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:08:33 PM</t>
+  </si>
+  <si>
+    <t> | 21 min | 1:41 PM—2:02 PM | Green Line | 1:41 PM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 25 min | 8.0 km | via Beleghata Main Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>4 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.19x</t>
+  </si>
+  <si>
+    <t>16.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:09:06 PM</t>
+  </si>
+  <si>
+    <t> | 9 min | 1:32 PM—1:41 PM | Green Line | 1:32 PM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 43 min | 7.2 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>34 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>4.78x</t>
+  </si>
+  <si>
+    <t>79.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:09:38 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 1:44 PM—2:02 PM | Green Line | 1:44 PM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 18 min | 4.9 km | via Narkeldanga Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:10:10 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 1:32 PM—1:44 PM | Green Line | 1:32 PM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 42 min | 7.6 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>30 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>3.50x</t>
+  </si>
+  <si>
+    <t>71.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:10:43 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 1:37 PM—2:02 PM | Green Line | 1:37 PM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 31 min | 12.7 km | via Mayo Rd and Park St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:12:27 PM</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:14:09 PM</t>
+  </si>
+  <si>
+    <t> | 9 min | 4.4 km | via Bangaon - Kulpi Rd/Biswa Bangla Sarani/Eastern Metropolitan Bypass/Thakurnagar - Panchpota Rd | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:15:52 PM</t>
+  </si>
+  <si>
+    <t> | 19 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:16:24 PM</t>
+  </si>
+  <si>
+    <t> | 19 min | 3:00 PM—3:19 PM | Purple Line | 3:00 PM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 7.8 km | via NH 12 | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>9 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.47x</t>
+  </si>
+  <si>
+    <t>32.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-19/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:16:42 PM</t>
+  </si>
+  <si>
+    <t> | 54 min | 3.9 km | via NH 12</t>
+  </si>
+  <si>
+    <t> | 15 min | 3.7 km | via NH 12 | Fastest route, despite slowdown on NH 12 causing 6-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>39 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.28x</t>
+  </si>
+  <si>
+    <t>72.2% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-20/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:17:01 PM</t>
+  </si>
+  <si>
+    <t> | 13 min | 4.1 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>44 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.23x</t>
+  </si>
+  <si>
+    <t>77.2% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-21/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:18:43 PM</t>
+  </si>
+  <si>
+    <t> | 24 min | 6.5 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:19:02 PM</t>
+  </si>
+  <si>
+    <t> | 33 min | 2.4 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t> | 11 min | 2.4 km | via NH 12 | Fastest route, despite slowdown on NH 12 causing 6-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>22 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.33x</t>
+  </si>
+  <si>
+    <t>66.7% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-23/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 1:19:20 PM</t>
+  </si>
+  <si>
+    <t> | 22 min | 1.5 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t>19 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.14x</t>
+  </si>
+  <si>
+    <t>86.4% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-24/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -851,7 +1335,31 @@
     <t>12:00 AM Savings (%)</t>
   </si>
   <si>
-    <t/>
+    <t>1:00 PM Scraped At</t>
+  </si>
+  <si>
+    <t>1:00 PM Actual Metro</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Walk</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro (min)</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Route</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>1:00 PM Car (min)</t>
+  </si>
+  <si>
+    <t>1:00 PM Faster Mode</t>
+  </si>
+  <si>
+    <t>1:00 PM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -3395,10 +3903,2143 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>13.3</v>
+      </c>
+      <c r="K2" t="s">
+        <v>271</v>
+      </c>
+      <c r="L2" t="s">
+        <v>272</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2">
+        <v>30</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R2">
+        <v>63</v>
+      </c>
+      <c r="S2" t="s">
+        <v>274</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="U2" t="s">
+        <v>276</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" t="s">
+        <v>277</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.8</v>
+      </c>
+      <c r="J3">
+        <v>14.7</v>
+      </c>
+      <c r="K3" t="s">
+        <v>271</v>
+      </c>
+      <c r="L3" t="s">
+        <v>272</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3">
+        <v>33</v>
+      </c>
+      <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>281</v>
+      </c>
+      <c r="R3">
+        <v>69</v>
+      </c>
+      <c r="S3" t="s">
+        <v>282</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="U3" t="s">
+        <v>284</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>285</v>
+      </c>
+      <c r="X3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>286</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>3.8</v>
+      </c>
+      <c r="J4">
+        <v>4.1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>271</v>
+      </c>
+      <c r="L4" t="s">
+        <v>272</v>
+      </c>
+      <c r="M4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4">
+        <v>54</v>
+      </c>
+      <c r="P4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>289</v>
+      </c>
+      <c r="R4">
+        <v>23</v>
+      </c>
+      <c r="S4" t="s">
+        <v>290</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="U4" t="s">
+        <v>292</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="W4" t="s">
+        <v>293</v>
+      </c>
+      <c r="X4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>294</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>296</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>5.2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>271</v>
+      </c>
+      <c r="L5" t="s">
+        <v>272</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5">
+        <v>11</v>
+      </c>
+      <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>297</v>
+      </c>
+      <c r="R5">
+        <v>39</v>
+      </c>
+      <c r="S5" t="s">
+        <v>298</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="U5" t="s">
+        <v>300</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W5" t="s">
+        <v>301</v>
+      </c>
+      <c r="X5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>302</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>304</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>271</v>
+      </c>
+      <c r="L6" t="s">
+        <v>272</v>
+      </c>
+      <c r="M6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6">
+        <v>11</v>
+      </c>
+      <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>305</v>
+      </c>
+      <c r="R6">
+        <v>23</v>
+      </c>
+      <c r="S6" t="s">
+        <v>306</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="U6" t="s">
+        <v>284</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W6" t="s">
+        <v>285</v>
+      </c>
+      <c r="X6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>307</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>6.2</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>271</v>
+      </c>
+      <c r="L7" t="s">
+        <v>272</v>
+      </c>
+      <c r="M7" t="s">
+        <v>38</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>26</v>
+      </c>
+      <c r="P7" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>311</v>
+      </c>
+      <c r="R7">
+        <v>28</v>
+      </c>
+      <c r="S7" t="s">
+        <v>312</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="U7" t="s">
+        <v>313</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>314</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>315</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>317</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>8.3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>271</v>
+      </c>
+      <c r="L8" t="s">
+        <v>272</v>
+      </c>
+      <c r="M8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8">
+        <v>24</v>
+      </c>
+      <c r="P8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>318</v>
+      </c>
+      <c r="R8">
+        <v>35</v>
+      </c>
+      <c r="S8" t="s">
+        <v>319</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U8" t="s">
+        <v>320</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W8" t="s">
+        <v>321</v>
+      </c>
+      <c r="X8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>322</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>324</v>
+      </c>
+      <c r="D9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9">
+        <v>7.1</v>
+      </c>
+      <c r="J9">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="s">
+        <v>271</v>
+      </c>
+      <c r="L9" t="s">
+        <v>272</v>
+      </c>
+      <c r="M9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9">
+        <v>17</v>
+      </c>
+      <c r="P9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>325</v>
+      </c>
+      <c r="R9">
+        <v>29</v>
+      </c>
+      <c r="S9" t="s">
+        <v>326</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="U9" t="s">
+        <v>327</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W9" t="s">
+        <v>328</v>
+      </c>
+      <c r="X9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>329</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>331</v>
+      </c>
+      <c r="D10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>8.8</v>
+      </c>
+      <c r="J10">
+        <v>8.8</v>
+      </c>
+      <c r="K10" t="s">
+        <v>271</v>
+      </c>
+      <c r="L10" t="s">
+        <v>272</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10">
+        <v>16</v>
+      </c>
+      <c r="P10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>332</v>
+      </c>
+      <c r="R10">
+        <v>57</v>
+      </c>
+      <c r="S10" t="s">
+        <v>333</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="U10" t="s">
+        <v>335</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W10" t="s">
+        <v>336</v>
+      </c>
+      <c r="X10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>337</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>339</v>
+      </c>
+      <c r="D11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E11" t="s">
+        <v>129</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>130</v>
+      </c>
+      <c r="H11" t="s">
+        <v>131</v>
+      </c>
+      <c r="I11">
+        <v>14.2</v>
+      </c>
+      <c r="J11">
+        <v>12.9</v>
+      </c>
+      <c r="K11" t="s">
+        <v>271</v>
+      </c>
+      <c r="L11" t="s">
+        <v>272</v>
+      </c>
+      <c r="M11" t="s">
+        <v>132</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11">
+        <v>30</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>340</v>
+      </c>
+      <c r="R11">
+        <v>56</v>
+      </c>
+      <c r="S11" t="s">
+        <v>341</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="U11" t="s">
+        <v>343</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W11" t="s">
+        <v>344</v>
+      </c>
+      <c r="X11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>345</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>347</v>
+      </c>
+      <c r="D12" t="s">
+        <v>140</v>
+      </c>
+      <c r="E12" t="s">
+        <v>129</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>141</v>
+      </c>
+      <c r="H12" t="s">
+        <v>131</v>
+      </c>
+      <c r="I12">
+        <v>8.3</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>271</v>
+      </c>
+      <c r="L12" t="s">
+        <v>272</v>
+      </c>
+      <c r="M12" t="s">
+        <v>132</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12">
+        <v>21</v>
+      </c>
+      <c r="P12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>348</v>
+      </c>
+      <c r="R12">
+        <v>25</v>
+      </c>
+      <c r="S12" t="s">
+        <v>349</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="U12" t="s">
+        <v>351</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W12" t="s">
+        <v>352</v>
+      </c>
+      <c r="X12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>353</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>355</v>
+      </c>
+      <c r="D13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E13" t="s">
+        <v>129</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" t="s">
+        <v>141</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>7.2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>271</v>
+      </c>
+      <c r="L13" t="s">
+        <v>272</v>
+      </c>
+      <c r="M13" t="s">
+        <v>132</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13">
+        <v>9</v>
+      </c>
+      <c r="P13" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>356</v>
+      </c>
+      <c r="R13">
+        <v>43</v>
+      </c>
+      <c r="S13" t="s">
+        <v>357</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="U13" t="s">
+        <v>359</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W13" t="s">
+        <v>360</v>
+      </c>
+      <c r="X13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>361</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>363</v>
+      </c>
+      <c r="D14" t="s">
+        <v>160</v>
+      </c>
+      <c r="E14" t="s">
+        <v>129</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>161</v>
+      </c>
+      <c r="H14" t="s">
+        <v>131</v>
+      </c>
+      <c r="I14">
+        <v>6.6</v>
+      </c>
+      <c r="J14">
+        <v>4.9</v>
+      </c>
+      <c r="K14" t="s">
+        <v>271</v>
+      </c>
+      <c r="L14" t="s">
+        <v>272</v>
+      </c>
+      <c r="M14" t="s">
+        <v>132</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14">
+        <v>18</v>
+      </c>
+      <c r="P14" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>364</v>
+      </c>
+      <c r="R14">
+        <v>18</v>
+      </c>
+      <c r="S14" t="s">
+        <v>365</v>
+      </c>
+      <c r="T14" t="s">
+        <v>144</v>
+      </c>
+      <c r="U14" t="s">
+        <v>145</v>
+      </c>
+      <c r="V14" t="s">
+        <v>146</v>
+      </c>
+      <c r="W14" t="s">
+        <v>147</v>
+      </c>
+      <c r="X14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>366</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>368</v>
+      </c>
+      <c r="D15" t="s">
+        <v>171</v>
+      </c>
+      <c r="E15" t="s">
+        <v>129</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>130</v>
+      </c>
+      <c r="H15" t="s">
+        <v>161</v>
+      </c>
+      <c r="I15">
+        <v>7.7</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>271</v>
+      </c>
+      <c r="L15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15">
+        <v>12</v>
+      </c>
+      <c r="P15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>369</v>
+      </c>
+      <c r="R15">
+        <v>42</v>
+      </c>
+      <c r="S15" t="s">
+        <v>370</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="U15" t="s">
+        <v>372</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W15" t="s">
+        <v>373</v>
+      </c>
+      <c r="X15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>374</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>376</v>
+      </c>
+      <c r="D16" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" t="s">
+        <v>129</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>131</v>
+      </c>
+      <c r="I16">
+        <v>11.3</v>
+      </c>
+      <c r="J16">
+        <v>12.7</v>
+      </c>
+      <c r="K16" t="s">
+        <v>271</v>
+      </c>
+      <c r="L16" t="s">
+        <v>272</v>
+      </c>
+      <c r="M16" t="s">
+        <v>132</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16">
+        <v>25</v>
+      </c>
+      <c r="P16" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>377</v>
+      </c>
+      <c r="R16">
+        <v>31</v>
+      </c>
+      <c r="S16" t="s">
+        <v>378</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="U16" t="s">
+        <v>183</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" t="s">
+        <v>184</v>
+      </c>
+      <c r="X16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>379</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>381</v>
+      </c>
+      <c r="D17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E17" t="s">
+        <v>189</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" t="s">
+        <v>190</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>9.8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>271</v>
+      </c>
+      <c r="L17" t="s">
+        <v>272</v>
+      </c>
+      <c r="M17" t="s">
+        <v>38</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17" t="s">
+        <v>382</v>
+      </c>
+      <c r="P17" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17">
+        <v>21</v>
+      </c>
+      <c r="S17" t="s">
+        <v>193</v>
+      </c>
+      <c r="T17" t="s">
+        <v>38</v>
+      </c>
+      <c r="U17" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" t="s">
+        <v>38</v>
+      </c>
+      <c r="W17" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>384</v>
+      </c>
+      <c r="D18" t="s">
+        <v>200</v>
+      </c>
+      <c r="E18" t="s">
+        <v>189</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>201</v>
+      </c>
+      <c r="H18" t="s">
+        <v>190</v>
+      </c>
+      <c r="I18">
+        <v>4.4</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>271</v>
+      </c>
+      <c r="L18" t="s">
+        <v>272</v>
+      </c>
+      <c r="M18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18" t="s">
+        <v>382</v>
+      </c>
+      <c r="P18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R18">
+        <v>9</v>
+      </c>
+      <c r="S18" t="s">
+        <v>385</v>
+      </c>
+      <c r="T18" t="s">
+        <v>38</v>
+      </c>
+      <c r="U18" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" t="s">
+        <v>38</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>387</v>
+      </c>
+      <c r="D19" t="s">
+        <v>210</v>
+      </c>
+      <c r="E19" t="s">
+        <v>189</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" t="s">
+        <v>211</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>271</v>
+      </c>
+      <c r="L19" t="s">
+        <v>272</v>
+      </c>
+      <c r="M19" t="s">
+        <v>38</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19" t="s">
+        <v>382</v>
+      </c>
+      <c r="P19" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19">
+        <v>19</v>
+      </c>
+      <c r="S19" t="s">
+        <v>388</v>
+      </c>
+      <c r="T19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U19" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" t="s">
+        <v>38</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>390</v>
+      </c>
+      <c r="D20" t="s">
+        <v>217</v>
+      </c>
+      <c r="E20" t="s">
+        <v>218</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>219</v>
+      </c>
+      <c r="H20" t="s">
+        <v>220</v>
+      </c>
+      <c r="I20">
+        <v>8.6</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>271</v>
+      </c>
+      <c r="L20" t="s">
+        <v>272</v>
+      </c>
+      <c r="M20" t="s">
+        <v>221</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20">
+        <v>19</v>
+      </c>
+      <c r="P20" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>391</v>
+      </c>
+      <c r="R20">
+        <v>28</v>
+      </c>
+      <c r="S20" t="s">
+        <v>392</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="U20" t="s">
+        <v>394</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W20" t="s">
+        <v>395</v>
+      </c>
+      <c r="X20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>396</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>398</v>
+      </c>
+      <c r="D21" t="s">
+        <v>230</v>
+      </c>
+      <c r="E21" t="s">
+        <v>218</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>231</v>
+      </c>
+      <c r="H21" t="s">
+        <v>220</v>
+      </c>
+      <c r="I21">
+        <v>3.9</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>271</v>
+      </c>
+      <c r="L21" t="s">
+        <v>272</v>
+      </c>
+      <c r="M21" t="s">
+        <v>38</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21">
+        <v>54</v>
+      </c>
+      <c r="P21" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>399</v>
+      </c>
+      <c r="R21">
+        <v>15</v>
+      </c>
+      <c r="S21" t="s">
+        <v>400</v>
+      </c>
+      <c r="T21" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="U21" t="s">
+        <v>402</v>
+      </c>
+      <c r="V21" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="W21" t="s">
+        <v>403</v>
+      </c>
+      <c r="X21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>404</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>406</v>
+      </c>
+      <c r="D22" t="s">
+        <v>240</v>
+      </c>
+      <c r="E22" t="s">
+        <v>218</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>219</v>
+      </c>
+      <c r="H22" t="s">
+        <v>231</v>
+      </c>
+      <c r="I22">
+        <v>4.1</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>271</v>
+      </c>
+      <c r="L22" t="s">
+        <v>272</v>
+      </c>
+      <c r="M22" t="s">
+        <v>38</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22">
+        <v>57</v>
+      </c>
+      <c r="P22" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>241</v>
+      </c>
+      <c r="R22">
+        <v>13</v>
+      </c>
+      <c r="S22" t="s">
+        <v>407</v>
+      </c>
+      <c r="T22" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="U22" t="s">
+        <v>409</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="W22" t="s">
+        <v>410</v>
+      </c>
+      <c r="X22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>411</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>413</v>
+      </c>
+      <c r="D23" t="s">
+        <v>249</v>
+      </c>
+      <c r="E23" t="s">
+        <v>218</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>219</v>
+      </c>
+      <c r="H23" t="s">
+        <v>250</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>271</v>
+      </c>
+      <c r="L23" t="s">
+        <v>272</v>
+      </c>
+      <c r="M23" t="s">
+        <v>38</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23" t="s">
+        <v>382</v>
+      </c>
+      <c r="P23" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>38</v>
+      </c>
+      <c r="R23">
+        <v>24</v>
+      </c>
+      <c r="S23" t="s">
+        <v>414</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" t="s">
+        <v>38</v>
+      </c>
+      <c r="W23" t="s">
+        <v>38</v>
+      </c>
+      <c r="X23" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>416</v>
+      </c>
+      <c r="D24" t="s">
+        <v>258</v>
+      </c>
+      <c r="E24" t="s">
+        <v>218</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>231</v>
+      </c>
+      <c r="H24" t="s">
+        <v>250</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>271</v>
+      </c>
+      <c r="L24" t="s">
+        <v>272</v>
+      </c>
+      <c r="M24" t="s">
+        <v>38</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24">
+        <v>33</v>
+      </c>
+      <c r="P24" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>417</v>
+      </c>
+      <c r="R24">
+        <v>11</v>
+      </c>
+      <c r="S24" t="s">
+        <v>418</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="U24" t="s">
+        <v>420</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="W24" t="s">
+        <v>421</v>
+      </c>
+      <c r="X24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>422</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>424</v>
+      </c>
+      <c r="D25" t="s">
+        <v>265</v>
+      </c>
+      <c r="E25" t="s">
+        <v>218</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>250</v>
+      </c>
+      <c r="H25" t="s">
+        <v>220</v>
+      </c>
+      <c r="I25">
+        <v>1.5</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>271</v>
+      </c>
+      <c r="L25" t="s">
+        <v>272</v>
+      </c>
+      <c r="M25" t="s">
+        <v>38</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25">
+        <v>22</v>
+      </c>
+      <c r="P25" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>425</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s">
+        <v>267</v>
+      </c>
+      <c r="T25" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="U25" t="s">
+        <v>427</v>
+      </c>
+      <c r="V25" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="W25" t="s">
+        <v>428</v>
+      </c>
+      <c r="X25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>429</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>430</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1"/>
+    <hyperlink ref="Y2" r:id="rId2"/>
+    <hyperlink ref="X3" r:id="rId3"/>
+    <hyperlink ref="Y3" r:id="rId4"/>
+    <hyperlink ref="X4" r:id="rId5"/>
+    <hyperlink ref="Y4" r:id="rId6"/>
+    <hyperlink ref="X5" r:id="rId7"/>
+    <hyperlink ref="Y5" r:id="rId8"/>
+    <hyperlink ref="X6" r:id="rId9"/>
+    <hyperlink ref="Y6" r:id="rId10"/>
+    <hyperlink ref="X7" r:id="rId11"/>
+    <hyperlink ref="Y7" r:id="rId12"/>
+    <hyperlink ref="X8" r:id="rId13"/>
+    <hyperlink ref="Y8" r:id="rId14"/>
+    <hyperlink ref="X9" r:id="rId15"/>
+    <hyperlink ref="Y9" r:id="rId16"/>
+    <hyperlink ref="X10" r:id="rId17"/>
+    <hyperlink ref="Y10" r:id="rId18"/>
+    <hyperlink ref="X11" r:id="rId19"/>
+    <hyperlink ref="Y11" r:id="rId20"/>
+    <hyperlink ref="X12" r:id="rId21"/>
+    <hyperlink ref="Y12" r:id="rId22"/>
+    <hyperlink ref="X13" r:id="rId23"/>
+    <hyperlink ref="Y13" r:id="rId24"/>
+    <hyperlink ref="X14" r:id="rId25"/>
+    <hyperlink ref="Y14" r:id="rId26"/>
+    <hyperlink ref="X15" r:id="rId27"/>
+    <hyperlink ref="Y15" r:id="rId28"/>
+    <hyperlink ref="X16" r:id="rId29"/>
+    <hyperlink ref="Y16" r:id="rId30"/>
+    <hyperlink ref="Y17" r:id="rId31"/>
+    <hyperlink ref="Y18" r:id="rId32"/>
+    <hyperlink ref="Y19" r:id="rId33"/>
+    <hyperlink ref="X20" r:id="rId34"/>
+    <hyperlink ref="Y20" r:id="rId35"/>
+    <hyperlink ref="X21" r:id="rId36"/>
+    <hyperlink ref="Y21" r:id="rId37"/>
+    <hyperlink ref="X22" r:id="rId38"/>
+    <hyperlink ref="Y22" r:id="rId39"/>
+    <hyperlink ref="Y23" r:id="rId40"/>
+    <hyperlink ref="X24" r:id="rId41"/>
+    <hyperlink ref="Y24" r:id="rId42"/>
+    <hyperlink ref="X25" r:id="rId43"/>
+    <hyperlink ref="Y25" r:id="rId44"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -3418,34 +6059,61 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>270</v>
+        <v>431</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>271</v>
+        <v>432</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>272</v>
+        <v>433</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>273</v>
+        <v>434</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>274</v>
+        <v>435</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>275</v>
+        <v>436</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>276</v>
+        <v>437</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>277</v>
+        <v>438</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>278</v>
+        <v>439</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>448</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -3491,8 +6159,35 @@
       <c r="O2" t="s">
         <v>44</v>
       </c>
+      <c r="P2" t="s">
+        <v>270</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2">
+        <v>30</v>
+      </c>
+      <c r="T2" t="s">
+        <v>39</v>
+      </c>
+      <c r="U2" t="s">
+        <v>273</v>
+      </c>
+      <c r="V2">
+        <v>63</v>
+      </c>
+      <c r="W2" t="s">
+        <v>39</v>
+      </c>
+      <c r="X2" t="s">
+        <v>277</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -3538,8 +6233,35 @@
       <c r="O3" t="s">
         <v>55</v>
       </c>
+      <c r="P3" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>38</v>
+      </c>
+      <c r="S3">
+        <v>33</v>
+      </c>
+      <c r="T3" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3" t="s">
+        <v>281</v>
+      </c>
+      <c r="V3">
+        <v>69</v>
+      </c>
+      <c r="W3" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3" t="s">
+        <v>285</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -3585,8 +6307,35 @@
       <c r="O4" t="s">
         <v>67</v>
       </c>
+      <c r="P4" t="s">
+        <v>288</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R4" t="s">
+        <v>38</v>
+      </c>
+      <c r="S4">
+        <v>54</v>
+      </c>
+      <c r="T4" t="s">
+        <v>382</v>
+      </c>
+      <c r="U4" t="s">
+        <v>289</v>
+      </c>
+      <c r="V4">
+        <v>23</v>
+      </c>
+      <c r="W4" t="s">
+        <v>166</v>
+      </c>
+      <c r="X4" t="s">
+        <v>293</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -3632,8 +6381,35 @@
       <c r="O5" t="s">
         <v>76</v>
       </c>
+      <c r="P5" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R5" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5">
+        <v>11</v>
+      </c>
+      <c r="T5" t="s">
+        <v>39</v>
+      </c>
+      <c r="U5" t="s">
+        <v>297</v>
+      </c>
+      <c r="V5">
+        <v>39</v>
+      </c>
+      <c r="W5" t="s">
+        <v>39</v>
+      </c>
+      <c r="X5" t="s">
+        <v>301</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -3679,8 +6455,35 @@
       <c r="O6" t="s">
         <v>86</v>
       </c>
+      <c r="P6" t="s">
+        <v>304</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S6">
+        <v>11</v>
+      </c>
+      <c r="T6" t="s">
+        <v>39</v>
+      </c>
+      <c r="U6" t="s">
+        <v>305</v>
+      </c>
+      <c r="V6">
+        <v>23</v>
+      </c>
+      <c r="W6" t="s">
+        <v>39</v>
+      </c>
+      <c r="X6" t="s">
+        <v>285</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -3726,8 +6529,35 @@
       <c r="O7" t="s">
         <v>95</v>
       </c>
+      <c r="P7" t="s">
+        <v>309</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>38</v>
+      </c>
+      <c r="R7" t="s">
+        <v>38</v>
+      </c>
+      <c r="S7">
+        <v>26</v>
+      </c>
+      <c r="T7" t="s">
+        <v>310</v>
+      </c>
+      <c r="U7" t="s">
+        <v>311</v>
+      </c>
+      <c r="V7">
+        <v>28</v>
+      </c>
+      <c r="W7" t="s">
+        <v>39</v>
+      </c>
+      <c r="X7" t="s">
+        <v>314</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -3773,8 +6603,35 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
+      <c r="P8" t="s">
+        <v>317</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>37</v>
+      </c>
+      <c r="R8" t="s">
+        <v>38</v>
+      </c>
+      <c r="S8">
+        <v>24</v>
+      </c>
+      <c r="T8" t="s">
+        <v>39</v>
+      </c>
+      <c r="U8" t="s">
+        <v>318</v>
+      </c>
+      <c r="V8">
+        <v>35</v>
+      </c>
+      <c r="W8" t="s">
+        <v>39</v>
+      </c>
+      <c r="X8" t="s">
+        <v>321</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -3820,8 +6677,35 @@
       <c r="O9" t="s">
         <v>115</v>
       </c>
+      <c r="P9" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>37</v>
+      </c>
+      <c r="R9" t="s">
+        <v>38</v>
+      </c>
+      <c r="S9">
+        <v>17</v>
+      </c>
+      <c r="T9" t="s">
+        <v>39</v>
+      </c>
+      <c r="U9" t="s">
+        <v>325</v>
+      </c>
+      <c r="V9">
+        <v>29</v>
+      </c>
+      <c r="W9" t="s">
+        <v>39</v>
+      </c>
+      <c r="X9" t="s">
+        <v>328</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>119</v>
       </c>
@@ -3867,8 +6751,35 @@
       <c r="O10" t="s">
         <v>124</v>
       </c>
+      <c r="P10" t="s">
+        <v>331</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>37</v>
+      </c>
+      <c r="R10" t="s">
+        <v>38</v>
+      </c>
+      <c r="S10">
+        <v>16</v>
+      </c>
+      <c r="T10" t="s">
+        <v>39</v>
+      </c>
+      <c r="U10" t="s">
+        <v>332</v>
+      </c>
+      <c r="V10">
+        <v>57</v>
+      </c>
+      <c r="W10" t="s">
+        <v>39</v>
+      </c>
+      <c r="X10" t="s">
+        <v>336</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>128</v>
       </c>
@@ -3914,8 +6825,35 @@
       <c r="O11" t="s">
         <v>136</v>
       </c>
+      <c r="P11" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>132</v>
+      </c>
+      <c r="R11" t="s">
+        <v>38</v>
+      </c>
+      <c r="S11">
+        <v>30</v>
+      </c>
+      <c r="T11" t="s">
+        <v>39</v>
+      </c>
+      <c r="U11" t="s">
+        <v>340</v>
+      </c>
+      <c r="V11">
+        <v>56</v>
+      </c>
+      <c r="W11" t="s">
+        <v>39</v>
+      </c>
+      <c r="X11" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>140</v>
       </c>
@@ -3961,8 +6899,35 @@
       <c r="O12" t="s">
         <v>147</v>
       </c>
+      <c r="P12" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>132</v>
+      </c>
+      <c r="R12" t="s">
+        <v>38</v>
+      </c>
+      <c r="S12">
+        <v>21</v>
+      </c>
+      <c r="T12" t="s">
+        <v>39</v>
+      </c>
+      <c r="U12" t="s">
+        <v>348</v>
+      </c>
+      <c r="V12">
+        <v>25</v>
+      </c>
+      <c r="W12" t="s">
+        <v>39</v>
+      </c>
+      <c r="X12" t="s">
+        <v>352</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>151</v>
       </c>
@@ -4008,8 +6973,35 @@
       <c r="O13" t="s">
         <v>156</v>
       </c>
+      <c r="P13" t="s">
+        <v>355</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>132</v>
+      </c>
+      <c r="R13" t="s">
+        <v>38</v>
+      </c>
+      <c r="S13">
+        <v>9</v>
+      </c>
+      <c r="T13" t="s">
+        <v>39</v>
+      </c>
+      <c r="U13" t="s">
+        <v>356</v>
+      </c>
+      <c r="V13">
+        <v>43</v>
+      </c>
+      <c r="W13" t="s">
+        <v>39</v>
+      </c>
+      <c r="X13" t="s">
+        <v>360</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>160</v>
       </c>
@@ -4055,8 +7047,35 @@
       <c r="O14" t="s">
         <v>167</v>
       </c>
+      <c r="P14" t="s">
+        <v>363</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>132</v>
+      </c>
+      <c r="R14" t="s">
+        <v>38</v>
+      </c>
+      <c r="S14">
+        <v>18</v>
+      </c>
+      <c r="T14" t="s">
+        <v>39</v>
+      </c>
+      <c r="U14" t="s">
+        <v>364</v>
+      </c>
+      <c r="V14">
+        <v>18</v>
+      </c>
+      <c r="W14" t="s">
+        <v>146</v>
+      </c>
+      <c r="X14" t="s">
+        <v>147</v>
+      </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>171</v>
       </c>
@@ -4102,8 +7121,35 @@
       <c r="O15" t="s">
         <v>175</v>
       </c>
+      <c r="P15" t="s">
+        <v>368</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>132</v>
+      </c>
+      <c r="R15" t="s">
+        <v>38</v>
+      </c>
+      <c r="S15">
+        <v>12</v>
+      </c>
+      <c r="T15" t="s">
+        <v>39</v>
+      </c>
+      <c r="U15" t="s">
+        <v>369</v>
+      </c>
+      <c r="V15">
+        <v>42</v>
+      </c>
+      <c r="W15" t="s">
+        <v>39</v>
+      </c>
+      <c r="X15" t="s">
+        <v>373</v>
+      </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>179</v>
       </c>
@@ -4149,8 +7195,35 @@
       <c r="O16" t="s">
         <v>184</v>
       </c>
+      <c r="P16" t="s">
+        <v>376</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>132</v>
+      </c>
+      <c r="R16" t="s">
+        <v>38</v>
+      </c>
+      <c r="S16">
+        <v>25</v>
+      </c>
+      <c r="T16" t="s">
+        <v>39</v>
+      </c>
+      <c r="U16" t="s">
+        <v>377</v>
+      </c>
+      <c r="V16">
+        <v>31</v>
+      </c>
+      <c r="W16" t="s">
+        <v>39</v>
+      </c>
+      <c r="X16" t="s">
+        <v>184</v>
+      </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>188</v>
       </c>
@@ -4196,8 +7269,35 @@
       <c r="O17" t="s">
         <v>196</v>
       </c>
+      <c r="P17" t="s">
+        <v>381</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17" t="s">
+        <v>38</v>
+      </c>
+      <c r="S17" t="s">
+        <v>382</v>
+      </c>
+      <c r="T17" t="s">
+        <v>38</v>
+      </c>
+      <c r="U17" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17">
+        <v>21</v>
+      </c>
+      <c r="W17" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>200</v>
       </c>
@@ -4243,8 +7343,35 @@
       <c r="O18" t="s">
         <v>206</v>
       </c>
+      <c r="P18" t="s">
+        <v>384</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R18" t="s">
+        <v>38</v>
+      </c>
+      <c r="S18" t="s">
+        <v>382</v>
+      </c>
+      <c r="T18" t="s">
+        <v>38</v>
+      </c>
+      <c r="U18" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18">
+        <v>9</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -4290,8 +7417,35 @@
       <c r="O19" t="s">
         <v>147</v>
       </c>
+      <c r="P19" t="s">
+        <v>387</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19" t="s">
+        <v>38</v>
+      </c>
+      <c r="S19" t="s">
+        <v>382</v>
+      </c>
+      <c r="T19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U19" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19">
+        <v>19</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>217</v>
       </c>
@@ -4337,8 +7491,35 @@
       <c r="O20" t="s">
         <v>226</v>
       </c>
+      <c r="P20" t="s">
+        <v>390</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>221</v>
+      </c>
+      <c r="R20" t="s">
+        <v>38</v>
+      </c>
+      <c r="S20">
+        <v>19</v>
+      </c>
+      <c r="T20" t="s">
+        <v>39</v>
+      </c>
+      <c r="U20" t="s">
+        <v>391</v>
+      </c>
+      <c r="V20">
+        <v>28</v>
+      </c>
+      <c r="W20" t="s">
+        <v>39</v>
+      </c>
+      <c r="X20" t="s">
+        <v>395</v>
+      </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>230</v>
       </c>
@@ -4384,8 +7565,35 @@
       <c r="O21" t="s">
         <v>236</v>
       </c>
+      <c r="P21" t="s">
+        <v>398</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>38</v>
+      </c>
+      <c r="R21" t="s">
+        <v>38</v>
+      </c>
+      <c r="S21">
+        <v>54</v>
+      </c>
+      <c r="T21" t="s">
+        <v>382</v>
+      </c>
+      <c r="U21" t="s">
+        <v>399</v>
+      </c>
+      <c r="V21">
+        <v>15</v>
+      </c>
+      <c r="W21" t="s">
+        <v>166</v>
+      </c>
+      <c r="X21" t="s">
+        <v>403</v>
+      </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>240</v>
       </c>
@@ -4417,7 +7625,7 @@
         <v>57</v>
       </c>
       <c r="K22" t="s">
-        <v>279</v>
+        <v>382</v>
       </c>
       <c r="L22" t="s">
         <v>241</v>
@@ -4431,8 +7639,35 @@
       <c r="O22" t="s">
         <v>245</v>
       </c>
+      <c r="P22" t="s">
+        <v>406</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>38</v>
+      </c>
+      <c r="R22" t="s">
+        <v>38</v>
+      </c>
+      <c r="S22">
+        <v>57</v>
+      </c>
+      <c r="T22" t="s">
+        <v>382</v>
+      </c>
+      <c r="U22" t="s">
+        <v>241</v>
+      </c>
+      <c r="V22">
+        <v>13</v>
+      </c>
+      <c r="W22" t="s">
+        <v>166</v>
+      </c>
+      <c r="X22" t="s">
+        <v>410</v>
+      </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>249</v>
       </c>
@@ -4478,8 +7713,35 @@
       <c r="O23" t="s">
         <v>254</v>
       </c>
+      <c r="P23" t="s">
+        <v>413</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>38</v>
+      </c>
+      <c r="R23" t="s">
+        <v>38</v>
+      </c>
+      <c r="S23" t="s">
+        <v>382</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23">
+        <v>24</v>
+      </c>
+      <c r="W23" t="s">
+        <v>38</v>
+      </c>
+      <c r="X23" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>258</v>
       </c>
@@ -4525,8 +7787,35 @@
       <c r="O24" t="s">
         <v>261</v>
       </c>
+      <c r="P24" t="s">
+        <v>416</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>38</v>
+      </c>
+      <c r="R24" t="s">
+        <v>38</v>
+      </c>
+      <c r="S24">
+        <v>33</v>
+      </c>
+      <c r="T24" t="s">
+        <v>382</v>
+      </c>
+      <c r="U24" t="s">
+        <v>417</v>
+      </c>
+      <c r="V24">
+        <v>11</v>
+      </c>
+      <c r="W24" t="s">
+        <v>166</v>
+      </c>
+      <c r="X24" t="s">
+        <v>421</v>
+      </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>265</v>
       </c>
@@ -4572,9 +7861,36 @@
       <c r="O25" t="s">
         <v>147</v>
       </c>
+      <c r="P25" t="s">
+        <v>424</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>38</v>
+      </c>
+      <c r="R25" t="s">
+        <v>38</v>
+      </c>
+      <c r="S25">
+        <v>22</v>
+      </c>
+      <c r="T25" t="s">
+        <v>382</v>
+      </c>
+      <c r="U25" t="s">
+        <v>425</v>
+      </c>
+      <c r="V25">
+        <v>3</v>
+      </c>
+      <c r="W25" t="s">
+        <v>166</v>
+      </c>
+      <c r="X25" t="s">
+        <v>428</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:X1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Auto-collect traffic data: 2026-10-17 07:42 PM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-10-17_Sat.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-10-17_Sat.xlsx
@@ -6,14 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="1_00 PM" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="7_00 PM" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="All Periods Combined" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2424" uniqueCount="532">
   <si>
     <t>Date</t>
   </si>
@@ -1308,6 +1309,228 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/1_00_PM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>10/17/2026, 7:04:36 PM</t>
+  </si>
+  <si>
+    <t>7:00 PM</t>
+  </si>
+  <si>
+    <t>Saturday (Weekend) - Evening Peak</t>
+  </si>
+  <si>
+    <t> | 1 hr 5 min | 14.1 km | via Barrackpore Trunk Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:06:19 PM</t>
+  </si>
+  <si>
+    <t> | 1 hr 13 min | 17.2 km | via Baghajatin Station Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:08:05 PM</t>
+  </si>
+  <si>
+    <t> | 27 min | 4.1 km | via Belgachia Rd/Khudiram Bose Sarani | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:09:47 PM</t>
+  </si>
+  <si>
+    <t> | 50 min | 5.7 km | via Bidhan Sarani Rd and Central Ave/Chittaranjan Ave | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:11:28 PM</t>
+  </si>
+  <si>
+    <t> | 26 min | 5.1 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:11:46 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:24 AM—7:42 AM | 32218 - Dankuni - Sealdah Local   | 7:27 AM from Dakshineswar 8 min late |  8 min | Details</t>
+  </si>
+  <si>
+    <t> | 29 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.61x</t>
+  </si>
+  <si>
+    <t>37.9% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:13:30 PM</t>
+  </si>
+  <si>
+    <t> | 40 min | 8.3 km | via Chowringee Rd/Jawaharlal Nehru Rd and Ashutosh Mukherjee Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:15:20 PM</t>
+  </si>
+  <si>
+    <t> | 37 min | 6.4 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:17:05 PM</t>
+  </si>
+  <si>
+    <t> | 1 hr 5 min | 9.5 km | via Raja Dinendra St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:18:50 PM</t>
+  </si>
+  <si>
+    <t> | 56 min | 12.0 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:20:34 PM</t>
+  </si>
+  <si>
+    <t> | 29 min | 8.0 km | via Beleghata Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:22:15 PM</t>
+  </si>
+  <si>
+    <t> | 45 min | 7.2 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:23:59 PM</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:25:44 PM</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:27:28 PM</t>
+  </si>
+  <si>
+    <t> | 39 min | 15.5 km | via AJC Bose Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:29:13 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 9.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:30:55 PM</t>
+  </si>
+  <si>
+    <t> | 10 min | 4.4 km | via Bangaon - Kulpi Rd/Biswa Bangla Sarani/Eastern Metropolitan Bypass/Thakurnagar - Panchpota Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:32:35 PM</t>
+  </si>
+  <si>
+    <t> | 23 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:34:18 PM</t>
+  </si>
+  <si>
+    <t> | 28 min | 7.8 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:36:00 PM</t>
+  </si>
+  <si>
+    <t> | 14 min | 3.7 km | via NH 12 | Fastest route, despite slowdown on NH 12 causing 6-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:37:44 PM</t>
+  </si>
+  <si>
+    <t> | 14 min | 4.1 km | via NH 12 | Fastest route, despite slowdown on NH 12 causing 5-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:39:25 PM</t>
+  </si>
+  <si>
+    <t> | 26 min | 6.5 km | via NH 12 | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:41:05 PM</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>10/17/2026, 7:42:47 PM</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-10-17/7_00_PM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -1360,6 +1583,33 @@
   </si>
   <si>
     <t>1:00 PM Savings (%)</t>
+  </si>
+  <si>
+    <t>7:00 PM Scraped At</t>
+  </si>
+  <si>
+    <t>7:00 PM Actual Metro</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Walk</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Route</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>7:00 PM Car (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Faster Mode</t>
+  </si>
+  <si>
+    <t>7:00 PM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -6036,10 +6286,2124 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>431</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>14.1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>432</v>
+      </c>
+      <c r="L2" t="s">
+        <v>433</v>
+      </c>
+      <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" t="s">
+        <v>382</v>
+      </c>
+      <c r="P2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2">
+        <v>65</v>
+      </c>
+      <c r="S2" t="s">
+        <v>434</v>
+      </c>
+      <c r="T2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" t="s">
+        <v>38</v>
+      </c>
+      <c r="W2" t="s">
+        <v>38</v>
+      </c>
+      <c r="X2" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>436</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.9</v>
+      </c>
+      <c r="J3">
+        <v>17.2</v>
+      </c>
+      <c r="K3" t="s">
+        <v>432</v>
+      </c>
+      <c r="L3" t="s">
+        <v>433</v>
+      </c>
+      <c r="M3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" t="s">
+        <v>382</v>
+      </c>
+      <c r="P3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>38</v>
+      </c>
+      <c r="R3">
+        <v>73</v>
+      </c>
+      <c r="S3" t="s">
+        <v>437</v>
+      </c>
+      <c r="T3" t="s">
+        <v>38</v>
+      </c>
+      <c r="U3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" t="s">
+        <v>38</v>
+      </c>
+      <c r="W3" t="s">
+        <v>38</v>
+      </c>
+      <c r="X3" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>3.8</v>
+      </c>
+      <c r="J4">
+        <v>4.1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>432</v>
+      </c>
+      <c r="L4" t="s">
+        <v>433</v>
+      </c>
+      <c r="M4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4" t="s">
+        <v>382</v>
+      </c>
+      <c r="P4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R4">
+        <v>27</v>
+      </c>
+      <c r="S4" t="s">
+        <v>440</v>
+      </c>
+      <c r="T4" t="s">
+        <v>38</v>
+      </c>
+      <c r="U4" t="s">
+        <v>38</v>
+      </c>
+      <c r="V4" t="s">
+        <v>38</v>
+      </c>
+      <c r="W4" t="s">
+        <v>38</v>
+      </c>
+      <c r="X4" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>442</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>5.7</v>
+      </c>
+      <c r="K5" t="s">
+        <v>432</v>
+      </c>
+      <c r="L5" t="s">
+        <v>433</v>
+      </c>
+      <c r="M5" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" t="s">
+        <v>382</v>
+      </c>
+      <c r="P5" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>38</v>
+      </c>
+      <c r="R5">
+        <v>50</v>
+      </c>
+      <c r="S5" t="s">
+        <v>443</v>
+      </c>
+      <c r="T5" t="s">
+        <v>38</v>
+      </c>
+      <c r="U5" t="s">
+        <v>38</v>
+      </c>
+      <c r="V5" t="s">
+        <v>38</v>
+      </c>
+      <c r="W5" t="s">
+        <v>38</v>
+      </c>
+      <c r="X5" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>445</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>432</v>
+      </c>
+      <c r="L6" t="s">
+        <v>433</v>
+      </c>
+      <c r="M6" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" t="s">
+        <v>382</v>
+      </c>
+      <c r="P6" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>38</v>
+      </c>
+      <c r="R6">
+        <v>26</v>
+      </c>
+      <c r="S6" t="s">
+        <v>446</v>
+      </c>
+      <c r="T6" t="s">
+        <v>38</v>
+      </c>
+      <c r="U6" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6" t="s">
+        <v>38</v>
+      </c>
+      <c r="W6" t="s">
+        <v>38</v>
+      </c>
+      <c r="X6" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>448</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>6.2</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>432</v>
+      </c>
+      <c r="L7" t="s">
+        <v>433</v>
+      </c>
+      <c r="M7" t="s">
+        <v>38</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>18</v>
+      </c>
+      <c r="P7" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>449</v>
+      </c>
+      <c r="R7">
+        <v>29</v>
+      </c>
+      <c r="S7" t="s">
+        <v>450</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U7" t="s">
+        <v>451</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>452</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>453</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>455</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>8.3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>432</v>
+      </c>
+      <c r="L8" t="s">
+        <v>433</v>
+      </c>
+      <c r="M8" t="s">
+        <v>38</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8" t="s">
+        <v>382</v>
+      </c>
+      <c r="P8" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>38</v>
+      </c>
+      <c r="R8">
+        <v>40</v>
+      </c>
+      <c r="S8" t="s">
+        <v>456</v>
+      </c>
+      <c r="T8" t="s">
+        <v>38</v>
+      </c>
+      <c r="U8" t="s">
+        <v>38</v>
+      </c>
+      <c r="V8" t="s">
+        <v>38</v>
+      </c>
+      <c r="W8" t="s">
+        <v>38</v>
+      </c>
+      <c r="X8" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>458</v>
+      </c>
+      <c r="D9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9">
+        <v>7.1</v>
+      </c>
+      <c r="J9">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="s">
+        <v>432</v>
+      </c>
+      <c r="L9" t="s">
+        <v>433</v>
+      </c>
+      <c r="M9" t="s">
+        <v>38</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9" t="s">
+        <v>382</v>
+      </c>
+      <c r="P9" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>38</v>
+      </c>
+      <c r="R9">
+        <v>37</v>
+      </c>
+      <c r="S9" t="s">
+        <v>459</v>
+      </c>
+      <c r="T9" t="s">
+        <v>38</v>
+      </c>
+      <c r="U9" t="s">
+        <v>38</v>
+      </c>
+      <c r="V9" t="s">
+        <v>38</v>
+      </c>
+      <c r="W9" t="s">
+        <v>38</v>
+      </c>
+      <c r="X9" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>461</v>
+      </c>
+      <c r="D10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>8.8</v>
+      </c>
+      <c r="J10">
+        <v>9.5</v>
+      </c>
+      <c r="K10" t="s">
+        <v>432</v>
+      </c>
+      <c r="L10" t="s">
+        <v>433</v>
+      </c>
+      <c r="M10" t="s">
+        <v>38</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10" t="s">
+        <v>382</v>
+      </c>
+      <c r="P10" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>38</v>
+      </c>
+      <c r="R10">
+        <v>65</v>
+      </c>
+      <c r="S10" t="s">
+        <v>462</v>
+      </c>
+      <c r="T10" t="s">
+        <v>38</v>
+      </c>
+      <c r="U10" t="s">
+        <v>38</v>
+      </c>
+      <c r="V10" t="s">
+        <v>38</v>
+      </c>
+      <c r="W10" t="s">
+        <v>38</v>
+      </c>
+      <c r="X10" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>464</v>
+      </c>
+      <c r="D11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E11" t="s">
+        <v>129</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>130</v>
+      </c>
+      <c r="H11" t="s">
+        <v>131</v>
+      </c>
+      <c r="I11">
+        <v>14.2</v>
+      </c>
+      <c r="J11">
+        <v>12</v>
+      </c>
+      <c r="K11" t="s">
+        <v>432</v>
+      </c>
+      <c r="L11" t="s">
+        <v>433</v>
+      </c>
+      <c r="M11" t="s">
+        <v>38</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11" t="s">
+        <v>382</v>
+      </c>
+      <c r="P11" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>38</v>
+      </c>
+      <c r="R11">
+        <v>56</v>
+      </c>
+      <c r="S11" t="s">
+        <v>465</v>
+      </c>
+      <c r="T11" t="s">
+        <v>38</v>
+      </c>
+      <c r="U11" t="s">
+        <v>38</v>
+      </c>
+      <c r="V11" t="s">
+        <v>38</v>
+      </c>
+      <c r="W11" t="s">
+        <v>38</v>
+      </c>
+      <c r="X11" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>467</v>
+      </c>
+      <c r="D12" t="s">
+        <v>140</v>
+      </c>
+      <c r="E12" t="s">
+        <v>129</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>141</v>
+      </c>
+      <c r="H12" t="s">
+        <v>131</v>
+      </c>
+      <c r="I12">
+        <v>8.6</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>432</v>
+      </c>
+      <c r="L12" t="s">
+        <v>433</v>
+      </c>
+      <c r="M12" t="s">
+        <v>38</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12" t="s">
+        <v>382</v>
+      </c>
+      <c r="P12" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>38</v>
+      </c>
+      <c r="R12">
+        <v>29</v>
+      </c>
+      <c r="S12" t="s">
+        <v>468</v>
+      </c>
+      <c r="T12" t="s">
+        <v>38</v>
+      </c>
+      <c r="U12" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12" t="s">
+        <v>38</v>
+      </c>
+      <c r="W12" t="s">
+        <v>38</v>
+      </c>
+      <c r="X12" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>470</v>
+      </c>
+      <c r="D13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E13" t="s">
+        <v>129</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" t="s">
+        <v>141</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>7.2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>432</v>
+      </c>
+      <c r="L13" t="s">
+        <v>433</v>
+      </c>
+      <c r="M13" t="s">
+        <v>38</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13" t="s">
+        <v>382</v>
+      </c>
+      <c r="P13" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>38</v>
+      </c>
+      <c r="R13">
+        <v>45</v>
+      </c>
+      <c r="S13" t="s">
+        <v>471</v>
+      </c>
+      <c r="T13" t="s">
+        <v>38</v>
+      </c>
+      <c r="U13" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13" t="s">
+        <v>38</v>
+      </c>
+      <c r="W13" t="s">
+        <v>38</v>
+      </c>
+      <c r="X13" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>473</v>
+      </c>
+      <c r="D14" t="s">
+        <v>160</v>
+      </c>
+      <c r="E14" t="s">
+        <v>129</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>161</v>
+      </c>
+      <c r="H14" t="s">
+        <v>131</v>
+      </c>
+      <c r="I14">
+        <v>6.6</v>
+      </c>
+      <c r="J14">
+        <v>4.9</v>
+      </c>
+      <c r="K14" t="s">
+        <v>432</v>
+      </c>
+      <c r="L14" t="s">
+        <v>433</v>
+      </c>
+      <c r="M14" t="s">
+        <v>38</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14" t="s">
+        <v>382</v>
+      </c>
+      <c r="P14" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>38</v>
+      </c>
+      <c r="R14">
+        <v>18</v>
+      </c>
+      <c r="S14" t="s">
+        <v>365</v>
+      </c>
+      <c r="T14" t="s">
+        <v>38</v>
+      </c>
+      <c r="U14" t="s">
+        <v>38</v>
+      </c>
+      <c r="V14" t="s">
+        <v>38</v>
+      </c>
+      <c r="W14" t="s">
+        <v>38</v>
+      </c>
+      <c r="X14" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>475</v>
+      </c>
+      <c r="D15" t="s">
+        <v>171</v>
+      </c>
+      <c r="E15" t="s">
+        <v>129</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>130</v>
+      </c>
+      <c r="H15" t="s">
+        <v>161</v>
+      </c>
+      <c r="I15">
+        <v>7.7</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>432</v>
+      </c>
+      <c r="L15" t="s">
+        <v>433</v>
+      </c>
+      <c r="M15" t="s">
+        <v>38</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15" t="s">
+        <v>382</v>
+      </c>
+      <c r="P15" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>38</v>
+      </c>
+      <c r="R15">
+        <v>42</v>
+      </c>
+      <c r="S15" t="s">
+        <v>370</v>
+      </c>
+      <c r="T15" t="s">
+        <v>38</v>
+      </c>
+      <c r="U15" t="s">
+        <v>38</v>
+      </c>
+      <c r="V15" t="s">
+        <v>38</v>
+      </c>
+      <c r="W15" t="s">
+        <v>38</v>
+      </c>
+      <c r="X15" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>477</v>
+      </c>
+      <c r="D16" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" t="s">
+        <v>129</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>131</v>
+      </c>
+      <c r="I16">
+        <v>11.3</v>
+      </c>
+      <c r="J16">
+        <v>15.5</v>
+      </c>
+      <c r="K16" t="s">
+        <v>432</v>
+      </c>
+      <c r="L16" t="s">
+        <v>433</v>
+      </c>
+      <c r="M16" t="s">
+        <v>38</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16" t="s">
+        <v>382</v>
+      </c>
+      <c r="P16" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>38</v>
+      </c>
+      <c r="R16">
+        <v>39</v>
+      </c>
+      <c r="S16" t="s">
+        <v>478</v>
+      </c>
+      <c r="T16" t="s">
+        <v>38</v>
+      </c>
+      <c r="U16" t="s">
+        <v>38</v>
+      </c>
+      <c r="V16" t="s">
+        <v>38</v>
+      </c>
+      <c r="W16" t="s">
+        <v>38</v>
+      </c>
+      <c r="X16" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>480</v>
+      </c>
+      <c r="D17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E17" t="s">
+        <v>189</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" t="s">
+        <v>190</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>9.8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>432</v>
+      </c>
+      <c r="L17" t="s">
+        <v>433</v>
+      </c>
+      <c r="M17" t="s">
+        <v>38</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17" t="s">
+        <v>382</v>
+      </c>
+      <c r="P17" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R17">
+        <v>25</v>
+      </c>
+      <c r="S17" t="s">
+        <v>481</v>
+      </c>
+      <c r="T17" t="s">
+        <v>38</v>
+      </c>
+      <c r="U17" t="s">
+        <v>38</v>
+      </c>
+      <c r="V17" t="s">
+        <v>38</v>
+      </c>
+      <c r="W17" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>483</v>
+      </c>
+      <c r="D18" t="s">
+        <v>200</v>
+      </c>
+      <c r="E18" t="s">
+        <v>189</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>201</v>
+      </c>
+      <c r="H18" t="s">
+        <v>190</v>
+      </c>
+      <c r="I18">
+        <v>4.4</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>432</v>
+      </c>
+      <c r="L18" t="s">
+        <v>433</v>
+      </c>
+      <c r="M18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18" t="s">
+        <v>382</v>
+      </c>
+      <c r="P18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R18">
+        <v>10</v>
+      </c>
+      <c r="S18" t="s">
+        <v>484</v>
+      </c>
+      <c r="T18" t="s">
+        <v>38</v>
+      </c>
+      <c r="U18" t="s">
+        <v>38</v>
+      </c>
+      <c r="V18" t="s">
+        <v>38</v>
+      </c>
+      <c r="W18" t="s">
+        <v>38</v>
+      </c>
+      <c r="X18" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>486</v>
+      </c>
+      <c r="D19" t="s">
+        <v>210</v>
+      </c>
+      <c r="E19" t="s">
+        <v>189</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" t="s">
+        <v>211</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>432</v>
+      </c>
+      <c r="L19" t="s">
+        <v>433</v>
+      </c>
+      <c r="M19" t="s">
+        <v>38</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19" t="s">
+        <v>382</v>
+      </c>
+      <c r="P19" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>38</v>
+      </c>
+      <c r="R19">
+        <v>23</v>
+      </c>
+      <c r="S19" t="s">
+        <v>487</v>
+      </c>
+      <c r="T19" t="s">
+        <v>38</v>
+      </c>
+      <c r="U19" t="s">
+        <v>38</v>
+      </c>
+      <c r="V19" t="s">
+        <v>38</v>
+      </c>
+      <c r="W19" t="s">
+        <v>38</v>
+      </c>
+      <c r="X19" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>489</v>
+      </c>
+      <c r="D20" t="s">
+        <v>217</v>
+      </c>
+      <c r="E20" t="s">
+        <v>218</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>219</v>
+      </c>
+      <c r="H20" t="s">
+        <v>220</v>
+      </c>
+      <c r="I20">
+        <v>7.9</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>432</v>
+      </c>
+      <c r="L20" t="s">
+        <v>433</v>
+      </c>
+      <c r="M20" t="s">
+        <v>38</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20" t="s">
+        <v>382</v>
+      </c>
+      <c r="P20" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>38</v>
+      </c>
+      <c r="R20">
+        <v>28</v>
+      </c>
+      <c r="S20" t="s">
+        <v>490</v>
+      </c>
+      <c r="T20" t="s">
+        <v>38</v>
+      </c>
+      <c r="U20" t="s">
+        <v>38</v>
+      </c>
+      <c r="V20" t="s">
+        <v>38</v>
+      </c>
+      <c r="W20" t="s">
+        <v>38</v>
+      </c>
+      <c r="X20" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>492</v>
+      </c>
+      <c r="D21" t="s">
+        <v>230</v>
+      </c>
+      <c r="E21" t="s">
+        <v>218</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>231</v>
+      </c>
+      <c r="H21" t="s">
+        <v>220</v>
+      </c>
+      <c r="I21">
+        <v>3.7</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>432</v>
+      </c>
+      <c r="L21" t="s">
+        <v>433</v>
+      </c>
+      <c r="M21" t="s">
+        <v>38</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21" t="s">
+        <v>382</v>
+      </c>
+      <c r="P21" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>38</v>
+      </c>
+      <c r="R21">
+        <v>14</v>
+      </c>
+      <c r="S21" t="s">
+        <v>493</v>
+      </c>
+      <c r="T21" t="s">
+        <v>38</v>
+      </c>
+      <c r="U21" t="s">
+        <v>38</v>
+      </c>
+      <c r="V21" t="s">
+        <v>38</v>
+      </c>
+      <c r="W21" t="s">
+        <v>38</v>
+      </c>
+      <c r="X21" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>495</v>
+      </c>
+      <c r="D22" t="s">
+        <v>240</v>
+      </c>
+      <c r="E22" t="s">
+        <v>218</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>219</v>
+      </c>
+      <c r="H22" t="s">
+        <v>231</v>
+      </c>
+      <c r="I22">
+        <v>4.2</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>432</v>
+      </c>
+      <c r="L22" t="s">
+        <v>433</v>
+      </c>
+      <c r="M22" t="s">
+        <v>38</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22" t="s">
+        <v>382</v>
+      </c>
+      <c r="P22" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>38</v>
+      </c>
+      <c r="R22">
+        <v>14</v>
+      </c>
+      <c r="S22" t="s">
+        <v>496</v>
+      </c>
+      <c r="T22" t="s">
+        <v>38</v>
+      </c>
+      <c r="U22" t="s">
+        <v>38</v>
+      </c>
+      <c r="V22" t="s">
+        <v>38</v>
+      </c>
+      <c r="W22" t="s">
+        <v>38</v>
+      </c>
+      <c r="X22" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>498</v>
+      </c>
+      <c r="D23" t="s">
+        <v>249</v>
+      </c>
+      <c r="E23" t="s">
+        <v>218</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>219</v>
+      </c>
+      <c r="H23" t="s">
+        <v>250</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>432</v>
+      </c>
+      <c r="L23" t="s">
+        <v>433</v>
+      </c>
+      <c r="M23" t="s">
+        <v>38</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23" t="s">
+        <v>382</v>
+      </c>
+      <c r="P23" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>38</v>
+      </c>
+      <c r="R23">
+        <v>26</v>
+      </c>
+      <c r="S23" t="s">
+        <v>499</v>
+      </c>
+      <c r="T23" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" t="s">
+        <v>38</v>
+      </c>
+      <c r="V23" t="s">
+        <v>38</v>
+      </c>
+      <c r="W23" t="s">
+        <v>38</v>
+      </c>
+      <c r="X23" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>501</v>
+      </c>
+      <c r="D24" t="s">
+        <v>258</v>
+      </c>
+      <c r="E24" t="s">
+        <v>218</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>231</v>
+      </c>
+      <c r="H24" t="s">
+        <v>250</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>432</v>
+      </c>
+      <c r="L24" t="s">
+        <v>433</v>
+      </c>
+      <c r="M24" t="s">
+        <v>38</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24" t="s">
+        <v>382</v>
+      </c>
+      <c r="P24" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>38</v>
+      </c>
+      <c r="R24">
+        <v>11</v>
+      </c>
+      <c r="S24" t="s">
+        <v>418</v>
+      </c>
+      <c r="T24" t="s">
+        <v>38</v>
+      </c>
+      <c r="U24" t="s">
+        <v>38</v>
+      </c>
+      <c r="V24" t="s">
+        <v>38</v>
+      </c>
+      <c r="W24" t="s">
+        <v>38</v>
+      </c>
+      <c r="X24" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>503</v>
+      </c>
+      <c r="D25" t="s">
+        <v>265</v>
+      </c>
+      <c r="E25" t="s">
+        <v>218</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>250</v>
+      </c>
+      <c r="H25" t="s">
+        <v>220</v>
+      </c>
+      <c r="I25">
+        <v>1.3</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>432</v>
+      </c>
+      <c r="L25" t="s">
+        <v>433</v>
+      </c>
+      <c r="M25" t="s">
+        <v>38</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25" t="s">
+        <v>382</v>
+      </c>
+      <c r="P25" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>38</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s">
+        <v>267</v>
+      </c>
+      <c r="T25" t="s">
+        <v>38</v>
+      </c>
+      <c r="U25" t="s">
+        <v>38</v>
+      </c>
+      <c r="V25" t="s">
+        <v>38</v>
+      </c>
+      <c r="W25" t="s">
+        <v>38</v>
+      </c>
+      <c r="X25" t="s">
+        <v>382</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>382</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>504</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="Y2" r:id="rId1"/>
+    <hyperlink ref="Y3" r:id="rId2"/>
+    <hyperlink ref="Y4" r:id="rId3"/>
+    <hyperlink ref="Y5" r:id="rId4"/>
+    <hyperlink ref="Y6" r:id="rId5"/>
+    <hyperlink ref="X7" r:id="rId6"/>
+    <hyperlink ref="Y7" r:id="rId7"/>
+    <hyperlink ref="Y8" r:id="rId8"/>
+    <hyperlink ref="Y9" r:id="rId9"/>
+    <hyperlink ref="Y10" r:id="rId10"/>
+    <hyperlink ref="Y11" r:id="rId11"/>
+    <hyperlink ref="Y12" r:id="rId12"/>
+    <hyperlink ref="Y13" r:id="rId13"/>
+    <hyperlink ref="Y14" r:id="rId14"/>
+    <hyperlink ref="Y15" r:id="rId15"/>
+    <hyperlink ref="Y16" r:id="rId16"/>
+    <hyperlink ref="Y17" r:id="rId17"/>
+    <hyperlink ref="Y18" r:id="rId18"/>
+    <hyperlink ref="Y19" r:id="rId19"/>
+    <hyperlink ref="Y20" r:id="rId20"/>
+    <hyperlink ref="Y21" r:id="rId21"/>
+    <hyperlink ref="Y22" r:id="rId22"/>
+    <hyperlink ref="Y23" r:id="rId23"/>
+    <hyperlink ref="Y24" r:id="rId24"/>
+    <hyperlink ref="Y25" r:id="rId25"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AG25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:33" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -6059,61 +8423,88 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>431</v>
+        <v>505</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>432</v>
+        <v>506</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>433</v>
+        <v>507</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>434</v>
+        <v>508</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>435</v>
+        <v>509</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>436</v>
+        <v>510</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>437</v>
+        <v>511</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>438</v>
+        <v>512</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>439</v>
+        <v>513</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>440</v>
+        <v>514</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>441</v>
+        <v>515</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>442</v>
+        <v>516</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>443</v>
+        <v>517</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>444</v>
+        <v>518</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>445</v>
+        <v>519</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>446</v>
+        <v>520</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>447</v>
+        <v>521</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>448</v>
+        <v>522</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="AD1" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="AE1" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="AF1" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="AG1" s="4" t="s">
+        <v>531</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -6186,8 +8577,35 @@
       <c r="X2" t="s">
         <v>277</v>
       </c>
+      <c r="Y2" t="s">
+        <v>431</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE2">
+        <v>65</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -6260,8 +8678,35 @@
       <c r="X3" t="s">
         <v>285</v>
       </c>
+      <c r="Y3" t="s">
+        <v>436</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE3">
+        <v>73</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -6334,8 +8779,35 @@
       <c r="X4" t="s">
         <v>293</v>
       </c>
+      <c r="Y4" t="s">
+        <v>439</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE4">
+        <v>27</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -6408,8 +8880,35 @@
       <c r="X5" t="s">
         <v>301</v>
       </c>
+      <c r="Y5" t="s">
+        <v>442</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE5">
+        <v>50</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -6482,8 +8981,35 @@
       <c r="X6" t="s">
         <v>285</v>
       </c>
+      <c r="Y6" t="s">
+        <v>445</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE6">
+        <v>26</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -6556,8 +9082,35 @@
       <c r="X7" t="s">
         <v>314</v>
       </c>
+      <c r="Y7" t="s">
+        <v>448</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB7">
+        <v>18</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>310</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>449</v>
+      </c>
+      <c r="AE7">
+        <v>29</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>452</v>
+      </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -6630,8 +9183,35 @@
       <c r="X8" t="s">
         <v>321</v>
       </c>
+      <c r="Y8" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE8">
+        <v>40</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -6704,8 +9284,35 @@
       <c r="X9" t="s">
         <v>328</v>
       </c>
+      <c r="Y9" t="s">
+        <v>458</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE9">
+        <v>37</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>119</v>
       </c>
@@ -6778,8 +9385,35 @@
       <c r="X10" t="s">
         <v>336</v>
       </c>
+      <c r="Y10" t="s">
+        <v>461</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE10">
+        <v>65</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>128</v>
       </c>
@@ -6852,8 +9486,35 @@
       <c r="X11" t="s">
         <v>344</v>
       </c>
+      <c r="Y11" t="s">
+        <v>464</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE11">
+        <v>56</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>140</v>
       </c>
@@ -6926,8 +9587,35 @@
       <c r="X12" t="s">
         <v>352</v>
       </c>
+      <c r="Y12" t="s">
+        <v>467</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE12">
+        <v>29</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>151</v>
       </c>
@@ -7000,8 +9688,35 @@
       <c r="X13" t="s">
         <v>360</v>
       </c>
+      <c r="Y13" t="s">
+        <v>470</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE13">
+        <v>45</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>160</v>
       </c>
@@ -7074,8 +9789,35 @@
       <c r="X14" t="s">
         <v>147</v>
       </c>
+      <c r="Y14" t="s">
+        <v>473</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE14">
+        <v>18</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>171</v>
       </c>
@@ -7148,8 +9890,35 @@
       <c r="X15" t="s">
         <v>373</v>
       </c>
+      <c r="Y15" t="s">
+        <v>475</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE15">
+        <v>42</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>179</v>
       </c>
@@ -7222,8 +9991,35 @@
       <c r="X16" t="s">
         <v>184</v>
       </c>
+      <c r="Y16" t="s">
+        <v>477</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE16">
+        <v>39</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>188</v>
       </c>
@@ -7296,8 +10092,35 @@
       <c r="X17" t="s">
         <v>38</v>
       </c>
+      <c r="Y17" t="s">
+        <v>480</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE17">
+        <v>25</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>200</v>
       </c>
@@ -7370,8 +10193,35 @@
       <c r="X18" t="s">
         <v>38</v>
       </c>
+      <c r="Y18" t="s">
+        <v>483</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE18">
+        <v>10</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -7444,8 +10294,35 @@
       <c r="X19" t="s">
         <v>38</v>
       </c>
+      <c r="Y19" t="s">
+        <v>486</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE19">
+        <v>23</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG19" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>217</v>
       </c>
@@ -7518,8 +10395,35 @@
       <c r="X20" t="s">
         <v>395</v>
       </c>
+      <c r="Y20" t="s">
+        <v>489</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE20">
+        <v>28</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>230</v>
       </c>
@@ -7592,8 +10496,35 @@
       <c r="X21" t="s">
         <v>403</v>
       </c>
+      <c r="Y21" t="s">
+        <v>492</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE21">
+        <v>14</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>240</v>
       </c>
@@ -7666,8 +10597,35 @@
       <c r="X22" t="s">
         <v>410</v>
       </c>
+      <c r="Y22" t="s">
+        <v>495</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE22">
+        <v>14</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>249</v>
       </c>
@@ -7740,8 +10698,35 @@
       <c r="X23" t="s">
         <v>38</v>
       </c>
+      <c r="Y23" t="s">
+        <v>498</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE23">
+        <v>26</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>258</v>
       </c>
@@ -7814,8 +10799,35 @@
       <c r="X24" t="s">
         <v>421</v>
       </c>
+      <c r="Y24" t="s">
+        <v>501</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE24">
+        <v>11</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>265</v>
       </c>
@@ -7888,9 +10900,36 @@
       <c r="X25" t="s">
         <v>428</v>
       </c>
+      <c r="Y25" t="s">
+        <v>503</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>382</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE25">
+        <v>3</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AG25" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1"/>
+  <autoFilter ref="A1:AG1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>